<commit_message>
fix(title): working title menu with quit sheet and focus handling
- Draw briefcase sheets in front, clipped by RectMask2D; add Quit sheet with confirm
- Fix TitleUI.Awake NRE via lazy TitleSheet.Button
- SequencePlayer.Stop with run id so the prologue does not leak past returning to title
- UIManager remembers and restores selection, disables input on covered pages
- Menu panel buttons no longer collapse to zero width
- Commit generated menu/notebook UI prefabs and Title scene (build index 0)

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Table/Excel/Text_UI.xlsx
+++ b/Table/Excel/Text_UI.xlsx
@@ -166,8 +166,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Text_UI" displayName="Text_UI" ref="B2:E42" headerRowCount="1" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="B2:E42"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Text_UI" displayName="Text_UI" ref="B2:E44" headerRowCount="1" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="B2:E44"/>
   <tableColumns count="4">
     <tableColumn id="1" name="DataId"/>
     <tableColumn id="2" name="Key" dataDxfId="3"/>
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E42"/>
+  <dimension ref="B2:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5" customHeight="1"/>
   <cols>
     <col width="3.125" customWidth="1" style="3" min="1" max="1"/>
@@ -1294,7 +1294,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="B42" t="n">
+      <c r="B42" s="0" t="n">
         <v>39</v>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -1310,6 +1310,46 @@
       <c r="E42" s="4" t="inlineStr">
         <is>
           <t>Need any help?</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="n">
+        <v>40</v>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>ui.title.quit</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>종료</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>Quit</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="n">
+        <v>41</v>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>ui.title.quit.confirm</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>게임을 종료할까요?</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>Quit the game?</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(table): validate command ids, text key refs, stale JSON; generate DataManager table list
- commandRefs check quest/note/sequence ids in Conditions and Actions (int ids compared as strings)
- refWhen: Sequence Param must be a Dialogue DataId when Type is dialogue
- TextKeyReferenceTests: @key refs in code/prefabs/scenes/assets exist; no Korean literals in localized Inspector fields
- Replace literal Inspector prompts/titles with Text keys
- RepoUpToDateTests: committed JSON and registry must match Excel
- Converter generates DataManager.Tables.cs (LoadSchemaTables)

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Table/Excel/Text_UI.xlsx
+++ b/Table/Excel/Text_UI.xlsx
@@ -166,8 +166,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Text_UI" displayName="Text_UI" ref="B2:E43" headerRowCount="1" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="B2:E43"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Text_UI" displayName="Text_UI" ref="B2:E45" headerRowCount="1" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="B2:E45"/>
   <tableColumns count="4">
     <tableColumn id="1" name="DataId"/>
     <tableColumn id="2" name="Key" dataDxfId="2"/>
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E44"/>
+  <dimension ref="B2:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5" customHeight="1"/>
   <cols>
     <col width="3.125" customWidth="1" style="3" min="1" max="1"/>
@@ -1334,10 +1334,36 @@
       </c>
     </row>
     <row r="44">
-      <c r="B44" s="0" t="n"/>
-      <c r="C44" s="4" t="n"/>
-      <c r="D44" s="4" t="n"/>
+      <c r="B44" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>ui.go_up</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>올라가기</t>
+        </is>
+      </c>
       <c r="E44" s="4" t="n"/>
+    </row>
+    <row r="45">
+      <c r="B45" t="n">
+        <v>43</v>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>ui.go_down</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>내려가기</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>